<commit_message>
añadido manual de implementacion
</commit_message>
<xml_diff>
--- a/01 Documentación/01.02 Analisis/EcoWaste PuntosFuncion.xlsx
+++ b/01 Documentación/01.02 Analisis/EcoWaste PuntosFuncion.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dbc_1\Documents\Desarrollo de software\proyecto\01 Documentación\01.02 Analisis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB229A6-25E7-4881-8A09-120FBD3ABAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A5523C-161F-470E-AA1B-0B40D3BAB49E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="16440" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DETALLE" sheetId="1" r:id="rId1"/>
     <sheet name="RESUMEN" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="Hoja1" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="128">
   <si>
     <t>ANÁLISIS DE PUNTOS DE FUNCIÓN — EcoWaste</t>
   </si>
@@ -82,19 +82,10 @@
     <t>EQ</t>
   </si>
   <si>
-    <t>Resumen</t>
-  </si>
-  <si>
     <t>ILF</t>
   </si>
   <si>
-    <t>Filas RF (azul): 10</t>
-  </si>
-  <si>
     <t>EIF</t>
-  </si>
-  <si>
-    <t>Sub-tareas: 26</t>
   </si>
   <si>
     <t>Resumen por tipo de función</t>
@@ -724,7 +715,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -787,6 +778,27 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -798,32 +810,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1105,12 +1093,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.25">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="2" spans="1:13" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="22"/>
@@ -1146,11 +1134,11 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
-        <v>23</v>
+      <c r="A3" s="26" t="s">
+        <v>20</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>10</v>
@@ -1183,9 +1171,9 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
+      <c r="A4" s="27"/>
       <c r="B4" s="12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>13</v>
@@ -1217,12 +1205,12 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="28"/>
+      <c r="A5" s="27"/>
       <c r="B5" s="12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>7</v>
@@ -1248,19 +1236,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
+      <c r="A6" s="29"/>
       <c r="B6" s="12"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
       <c r="E6" s="18"/>
-      <c r="G6" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="G6" s="5"/>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K6" s="3">
         <v>7</v>
@@ -1273,11 +1259,11 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>24</v>
+      <c r="A7" s="26" t="s">
+        <v>21</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>10</v>
@@ -1289,14 +1275,12 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G7" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="G7" s="6"/>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K7" s="3">
         <v>5</v>
@@ -1309,9 +1293,9 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="28"/>
+      <c r="A8" s="27"/>
       <c r="B8" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>13</v>
@@ -1323,20 +1307,18 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>18</v>
-      </c>
+      <c r="G8" s="6"/>
       <c r="H8">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="31"/>
+      <c r="A9" s="28"/>
       <c r="B9" s="12" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>7</v>
@@ -1351,11 +1333,11 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
-        <v>25</v>
+      <c r="A10" s="26" t="s">
+        <v>22</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>10</v>
@@ -1373,9 +1355,9 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28"/>
+      <c r="A11" s="27"/>
       <c r="B11" s="12" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>10</v>
@@ -1393,12 +1375,12 @@
       </c>
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28"/>
+      <c r="A12" s="27"/>
       <c r="B12" s="12" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>7</v>
@@ -1413,9 +1395,9 @@
       </c>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="28"/>
+      <c r="A13" s="27"/>
       <c r="B13" s="12" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>13</v>
@@ -1433,7 +1415,7 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
+      <c r="A14" s="29"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
@@ -1444,11 +1426,11 @@
       </c>
     </row>
     <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="23" t="s">
-        <v>26</v>
+      <c r="A15" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C15" s="14" t="s">
         <v>10</v>
@@ -1466,9 +1448,9 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="24"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>13</v>
@@ -1486,9 +1468,9 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="24"/>
+      <c r="A17" s="31"/>
       <c r="B17" s="12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>12</v>
@@ -1505,9 +1487,9 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="25"/>
+      <c r="A18" s="32"/>
       <c r="B18" s="17" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C18" s="17" t="s">
         <v>13</v>
@@ -1524,11 +1506,11 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="27" t="s">
-        <v>27</v>
+      <c r="A19" s="26" t="s">
+        <v>24</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>10</v>
@@ -1542,12 +1524,12 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="28"/>
+      <c r="A20" s="27"/>
       <c r="B20" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>7</v>
@@ -1561,9 +1543,9 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="31"/>
+      <c r="A21" s="28"/>
       <c r="B21" s="12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>12</v>
@@ -1572,7 +1554,7 @@
         <v>7</v>
       </c>
       <c r="E21" s="16">
-        <f>INDEX($K$3:$M$7,MATCH(C21,$J$3:$J$7,0),IF(UPPER(D21)="BAJA",1,IF(UPPER(D21)="MEDIA",2,3)))</f>
+        <f t="shared" ref="E21:E27" si="1">INDEX($K$3:$M$7,MATCH(C21,$J$3:$J$7,0),IF(UPPER(D21)="BAJA",1,IF(UPPER(D21)="MEDIA",2,3)))</f>
         <v>4</v>
       </c>
       <c r="H21">
@@ -1580,11 +1562,11 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="27" t="s">
-        <v>28</v>
+      <c r="A22" s="26" t="s">
+        <v>25</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C22" s="14" t="s">
         <v>10</v>
@@ -1593,7 +1575,7 @@
         <v>7</v>
       </c>
       <c r="E22" s="20">
-        <f>INDEX($K$3:$M$7,MATCH(C22,$J$3:$J$7,0),IF(UPPER(D22)="BAJA",1,IF(UPPER(D22)="MEDIA",2,3)))</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H22">
@@ -1601,9 +1583,9 @@
       </c>
     </row>
     <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28"/>
+      <c r="A23" s="27"/>
       <c r="B23" s="12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>13</v>
@@ -1612,7 +1594,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="19">
-        <f>INDEX($K$3:$M$7,MATCH(C23,$J$3:$J$7,0),IF(UPPER(D23)="BAJA",1,IF(UPPER(D23)="MEDIA",2,3)))</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H23">
@@ -1620,9 +1602,9 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="28"/>
+      <c r="A24" s="27"/>
       <c r="B24" s="12" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>13</v>
@@ -1631,7 +1613,7 @@
         <v>7</v>
       </c>
       <c r="E24" s="19">
-        <f>INDEX($K$3:$M$7,MATCH(C24,$J$3:$J$7,0),IF(UPPER(D24)="BAJA",1,IF(UPPER(D24)="MEDIA",2,3)))</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H24">
@@ -1639,9 +1621,9 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="28"/>
+      <c r="A25" s="27"/>
       <c r="B25" s="12" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>13</v>
@@ -1650,7 +1632,7 @@
         <v>8</v>
       </c>
       <c r="E25" s="16">
-        <f>INDEX($K$3:$M$7,MATCH(C25,$J$3:$J$7,0),IF(UPPER(D25)="BAJA",1,IF(UPPER(D25)="MEDIA",2,3)))</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="H25">
@@ -1658,9 +1640,9 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="32"/>
+      <c r="A26" s="29"/>
       <c r="B26" s="17" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C26" s="17" t="s">
         <v>12</v>
@@ -1669,7 +1651,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="18">
-        <f>INDEX($K$3:$M$7,MATCH(C26,$J$3:$J$7,0),IF(UPPER(D26)="BAJA",1,IF(UPPER(D26)="MEDIA",2,3)))</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="H26">
@@ -1677,20 +1659,20 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="27" t="s">
-        <v>29</v>
+      <c r="A27" s="26" t="s">
+        <v>26</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="C27" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="C27" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="35" t="s">
+      <c r="D27" s="12" t="s">
         <v>7</v>
       </c>
       <c r="E27" s="16">
-        <f>INDEX($K$3:$M$7,MATCH(C27,$J$3:$J$7,0),IF(UPPER(D27)="BAJA",1,IF(UPPER(D27)="MEDIA",2,3)))</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H27">
@@ -1698,9 +1680,9 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="28"/>
+      <c r="A28" s="27"/>
       <c r="B28" s="12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>13</v>
@@ -1717,9 +1699,9 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="28"/>
+      <c r="A29" s="27"/>
       <c r="B29" s="12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>13</v>
@@ -1736,9 +1718,9 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="28"/>
+      <c r="A30" s="27"/>
       <c r="B30" s="12" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>13</v>
@@ -1755,9 +1737,9 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="32"/>
+      <c r="A31" s="29"/>
       <c r="B31" s="12" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C31" s="17" t="s">
         <v>12</v>
@@ -1774,11 +1756,11 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="30" t="s">
-        <v>30</v>
+      <c r="A32" s="23" t="s">
+        <v>27</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C32" s="14" t="s">
         <v>10</v>
@@ -1795,12 +1777,12 @@
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="33"/>
+      <c r="A33" s="24"/>
       <c r="B33" s="12" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D33" s="12" t="s">
         <v>7</v>
@@ -1814,9 +1796,9 @@
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="33"/>
+      <c r="A34" s="24"/>
       <c r="B34" s="12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>13</v>
@@ -1833,9 +1815,9 @@
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="33"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C35" s="12" t="s">
         <v>12</v>
@@ -1852,12 +1834,12 @@
       </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="34"/>
+      <c r="A36" s="25"/>
       <c r="B36" s="17" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D36" s="17" t="s">
         <v>7</v>
@@ -1871,14 +1853,14 @@
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="30" t="s">
-        <v>31</v>
+      <c r="A37" s="23" t="s">
+        <v>28</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>7</v>
@@ -1892,9 +1874,9 @@
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="33"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="12" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C38" s="12" t="s">
         <v>13</v>
@@ -1911,9 +1893,9 @@
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="33"/>
+      <c r="A39" s="24"/>
       <c r="B39" s="12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C39" s="12" t="s">
         <v>12</v>
@@ -1930,28 +1912,28 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="33"/>
+      <c r="A40" s="24"/>
       <c r="B40" s="12" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C40" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E40" s="16">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="25"/>
+      <c r="B41" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="C41" s="17" t="s">
         <v>15</v>
-      </c>
-      <c r="D40" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E40" s="16">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="34"/>
-      <c r="B41" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="C41" s="17" t="s">
-        <v>17</v>
       </c>
       <c r="D41" s="17" t="s">
         <v>9</v>
@@ -1962,11 +1944,11 @@
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="30" t="s">
-        <v>32</v>
+      <c r="A42" s="23" t="s">
+        <v>29</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>10</v>
@@ -1980,12 +1962,12 @@
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="33"/>
+      <c r="A43" s="24"/>
       <c r="B43" s="12" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D43" s="12" t="s">
         <v>7</v>
@@ -1996,9 +1978,9 @@
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="33"/>
+      <c r="A44" s="24"/>
       <c r="B44" s="12" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C44" s="12" t="s">
         <v>13</v>
@@ -2012,12 +1994,12 @@
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="33"/>
+      <c r="A45" s="24"/>
       <c r="B45" s="12" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D45" s="12" t="s">
         <v>7</v>
@@ -2028,9 +2010,9 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="34"/>
+      <c r="A46" s="25"/>
       <c r="B46" s="17" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C46" s="17" t="s">
         <v>12</v>
@@ -2044,11 +2026,11 @@
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="30" t="s">
-        <v>33</v>
+      <c r="A47" s="23" t="s">
+        <v>30</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C47" s="14" t="s">
         <v>13</v>
@@ -2062,12 +2044,12 @@
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="33"/>
+      <c r="A48" s="24"/>
       <c r="B48" s="12" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D48" s="12" t="s">
         <v>7</v>
@@ -2078,9 +2060,9 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="33"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="12" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C49" s="12" t="s">
         <v>12</v>
@@ -2094,12 +2076,12 @@
       </c>
     </row>
     <row r="50" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="34"/>
+      <c r="A50" s="25"/>
       <c r="B50" s="17" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D50" s="17" t="s">
         <v>9</v>
@@ -2111,6 +2093,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A10:A14"/>
     <mergeCell ref="A42:A46"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="A32:A36"/>
@@ -2118,11 +2105,6 @@
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A22:A26"/>
     <mergeCell ref="A27:A31"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A10:A14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2140,25 +2122,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="A1" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2214,7 +2196,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="8" t="e">
         <f>COUNTIFS(DETALLE!$C$3:$C$32,A7,DETALLE!$H$3:$H$39,1)</f>
@@ -2231,7 +2213,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8" s="8" t="e">
         <f>COUNTIFS(DETALLE!$C$3:$C$32,A8,DETALLE!$H$3:$H$39,1)</f>
@@ -2259,7 +2241,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2284,33 +2266,33 @@
   <sheetData>
     <row r="3" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="11" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B4" s="12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>7</v>
@@ -2319,13 +2301,13 @@
     <row r="5" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B5" s="12"/>
       <c r="C5" s="12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>8</v>
@@ -2334,13 +2316,13 @@
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="12"/>
       <c r="C6" s="12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F6" s="12" t="s">
         <v>7</v>
@@ -2349,13 +2331,13 @@
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="12"/>
       <c r="C7" s="12" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>7</v>
@@ -2364,13 +2346,13 @@
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
       <c r="C8" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F8" s="12" t="s">
         <v>7</v>
@@ -2379,13 +2361,13 @@
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F9" s="12" t="s">
         <v>7</v>
@@ -2393,16 +2375,16 @@
     </row>
     <row r="10" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>7</v>
@@ -2411,13 +2393,13 @@
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>8</v>
@@ -2426,13 +2408,13 @@
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>7</v>
@@ -2441,13 +2423,13 @@
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F13" s="12" t="s">
         <v>7</v>
@@ -2456,13 +2438,13 @@
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F14" s="12" t="s">
         <v>7</v>
@@ -2471,13 +2453,13 @@
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12"/>
       <c r="C15" s="12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F15" s="12" t="s">
         <v>7</v>
@@ -2485,16 +2467,16 @@
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F16" s="12" t="s">
         <v>7</v>
@@ -2503,13 +2485,13 @@
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="12"/>
       <c r="C17" s="12" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>7</v>
@@ -2518,13 +2500,13 @@
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F18" s="12" t="s">
         <v>7</v>
@@ -2533,13 +2515,13 @@
     <row r="19" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B19" s="12"/>
       <c r="C19" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>8</v>
@@ -2548,13 +2530,13 @@
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="12"/>
       <c r="C20" s="12" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F20" s="12" t="s">
         <v>8</v>
@@ -2562,16 +2544,16 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F21" s="12" t="s">
         <v>7</v>
@@ -2580,13 +2562,13 @@
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="12"/>
       <c r="C22" s="12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F22" s="12" t="s">
         <v>8</v>
@@ -2595,13 +2577,13 @@
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="12"/>
       <c r="C23" s="12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F23" s="12" t="s">
         <v>8</v>
@@ -2610,13 +2592,13 @@
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="12"/>
       <c r="C24" s="12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F24" s="12" t="s">
         <v>7</v>
@@ -2624,16 +2606,16 @@
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F25" s="12" t="s">
         <v>7</v>
@@ -2642,13 +2624,13 @@
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="12"/>
       <c r="C26" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>7</v>
@@ -2657,13 +2639,13 @@
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F27" s="12" t="s">
         <v>7</v>
@@ -2672,13 +2654,13 @@
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="12"/>
       <c r="C28" s="12" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F28" s="12" t="s">
         <v>7</v>
@@ -2687,13 +2669,13 @@
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D29" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F29" s="12" t="s">
         <v>8</v>
@@ -2702,13 +2684,13 @@
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="12"/>
       <c r="C30" s="12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F30" s="12" t="s">
         <v>7</v>
@@ -2716,16 +2698,16 @@
     </row>
     <row r="31" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B31" s="12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F31" s="12" t="s">
         <v>7</v>
@@ -2734,13 +2716,13 @@
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="12"/>
       <c r="C32" s="12" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F32" s="12" t="s">
         <v>7</v>
@@ -2749,13 +2731,13 @@
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="12"/>
       <c r="C33" s="12" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D33" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F33" s="12" t="s">
         <v>8</v>
@@ -2764,13 +2746,13 @@
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="12"/>
       <c r="C34" s="12" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F34" s="12" t="s">
         <v>8</v>
@@ -2778,16 +2760,16 @@
     </row>
     <row r="35" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B35" s="12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D35" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F35" s="12" t="s">
         <v>7</v>
@@ -2796,13 +2778,13 @@
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D36" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F36" s="12" t="s">
         <v>7</v>
@@ -2811,13 +2793,13 @@
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" s="12"/>
       <c r="C37" s="12" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D37" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F37" s="12" t="s">
         <v>7</v>
@@ -2826,13 +2808,13 @@
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D38" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F38" s="12" t="s">
         <v>7</v>
@@ -2840,16 +2822,16 @@
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" s="12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F39" s="12" t="s">
         <v>7</v>
@@ -2858,13 +2840,13 @@
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" s="12"/>
       <c r="C40" s="12" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F40" s="12" t="s">
         <v>7</v>
@@ -2873,13 +2855,13 @@
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" s="12"/>
       <c r="C41" s="12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D41" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F41" s="12" t="s">
         <v>8</v>
@@ -2888,13 +2870,13 @@
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" s="12"/>
       <c r="C42" s="12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D42" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F42" s="12" t="s">
         <v>7</v>
@@ -2903,13 +2885,13 @@
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B43" s="12"/>
       <c r="C43" s="12" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F43" s="12" t="s">
         <v>7</v>
@@ -2917,16 +2899,16 @@
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B44" s="12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F44" s="12" t="s">
         <v>7</v>
@@ -2935,13 +2917,13 @@
     <row r="45" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B45" s="12"/>
       <c r="C45" s="12" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D45" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F45" s="12" t="s">
         <v>7</v>
@@ -2950,13 +2932,13 @@
     <row r="46" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B46" s="12"/>
       <c r="C46" s="12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D46" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F46" s="12" t="s">
         <v>7</v>
@@ -2965,13 +2947,13 @@
     <row r="47" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B47" s="12"/>
       <c r="C47" s="12" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F47" s="12" t="s">
         <v>7</v>
@@ -2980,13 +2962,13 @@
     <row r="48" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B48" s="12"/>
       <c r="C48" s="12" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F48" s="12" t="s">
         <v>9</v>
@@ -2994,16 +2976,16 @@
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B49" s="12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D49" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F49" s="12" t="s">
         <v>7</v>
@@ -3012,13 +2994,13 @@
     <row r="50" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B50" s="12"/>
       <c r="C50" s="12" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F50" s="12" t="s">
         <v>7</v>
@@ -3027,13 +3009,13 @@
     <row r="51" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B51" s="12"/>
       <c r="C51" s="12" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D51" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F51" s="12" t="s">
         <v>7</v>
@@ -3042,13 +3024,13 @@
     <row r="52" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B52" s="12"/>
       <c r="C52" s="12" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F52" s="12" t="s">
         <v>7</v>
@@ -3057,13 +3039,13 @@
     <row r="53" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B53" s="12"/>
       <c r="C53" s="12" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D53" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F53" s="12" t="s">
         <v>7</v>
@@ -3071,16 +3053,16 @@
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B54" s="12" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D54" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F54" s="12" t="s">
         <v>7</v>
@@ -3089,13 +3071,13 @@
     <row r="55" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B55" s="12"/>
       <c r="C55" s="12" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F55" s="12" t="s">
         <v>7</v>
@@ -3104,13 +3086,13 @@
     <row r="56" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B56" s="12"/>
       <c r="C56" s="12" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D56" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F56" s="12" t="s">
         <v>7</v>
@@ -3119,13 +3101,13 @@
     <row r="57" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B57" s="12"/>
       <c r="C57" s="12" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F57" s="12" t="s">
         <v>9</v>

</xml_diff>